<commit_message>
Restrurcturing and updating main.py
</commit_message>
<xml_diff>
--- a/params/Raw Parameters.xlsx
+++ b/params/Raw Parameters.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ce7bac70211bc540/Documents/Oxford 2025/03 Data/02 Irradiated/Refel FINAL/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ce7bac70211bc540/Documents/Git/raman-spectra-processing/params/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="218" documentId="8_{EDB9DC01-DA0F-4CF6-82DA-79403202B35E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5605A63-366E-442C-B973-A149E20E8450}"/>
+  <xr:revisionPtr revIDLastSave="220" documentId="8_{EDB9DC01-DA0F-4CF6-82DA-79403202B35E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DCB81A82-1D9D-431E-B248-EAD90E360E0D}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{175DB362-BC3B-4B7B-B945-DBED43F0BCFF}"/>
   </bookViews>
@@ -454,6 +454,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -466,20 +473,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="8">
     <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -491,7 +491,7 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -669,8 +669,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{88629AE6-1F5A-443C-A836-595CCA062C0C}" name="Location_1_graphite_peak_parameters14" displayName="Location_1_graphite_peak_parameters14" ref="U3:Z5" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="U3:Z5" xr:uid="{88629AE6-1F5A-443C-A836-595CCA062C0C}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{27F22DE0-B640-4AB6-872E-45C013ECFC2F}" uniqueName="1" name="Peak" queryTableFieldId="1" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{5D08E4F5-F578-4AC3-8363-12E0E74D580F}" uniqueName="2" name="Model" queryTableFieldId="2" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{27F22DE0-B640-4AB6-872E-45C013ECFC2F}" uniqueName="1" name="Peak" queryTableFieldId="1" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{5D08E4F5-F578-4AC3-8363-12E0E74D580F}" uniqueName="2" name="Model" queryTableFieldId="2" dataDxfId="3"/>
     <tableColumn id="3" xr3:uid="{9DF1D443-19CA-4526-BE48-04519F009B60}" uniqueName="3" name="Center (cm⁻¹)" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{EF63B764-2119-4267-81DD-692B0CD02703}" uniqueName="4" name="FWHM (cm⁻¹)" queryTableFieldId="4"/>
     <tableColumn id="5" xr3:uid="{16212206-06DE-4114-A459-5595F8CBE80C}" uniqueName="5" name="Area" queryTableFieldId="5"/>
@@ -685,7 +685,7 @@
   <autoFilter ref="B49:G67" xr:uid="{25938BD7-3BEC-4744-B44D-57F1C5BF2930}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{8E0C8E8D-A4D8-4F3F-A0D5-B3359A9FE231}" uniqueName="1" name="Peak" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{66EB0A78-9DD6-4490-93F6-D1373B4DDC18}" uniqueName="2" name="Model" queryTableFieldId="2" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{66EB0A78-9DD6-4490-93F6-D1373B4DDC18}" uniqueName="2" name="Model" queryTableFieldId="2" dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{95AC4A0F-4B08-4387-A2BD-E3382E431825}" uniqueName="3" name="Center (cm⁻¹)" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{BFEC92B1-6F43-4CB9-BE24-C4A025D3E542}" uniqueName="4" name="FWHM (cm⁻¹)" queryTableFieldId="4"/>
     <tableColumn id="5" xr3:uid="{C88BD2A1-C628-4EE3-80B5-1D79D1C23587}" uniqueName="5" name="Area" queryTableFieldId="5"/>
@@ -700,7 +700,7 @@
   <autoFilter ref="B71:G90" xr:uid="{0F98CC05-51BC-49C8-983A-CA804D806259}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{470EEF05-DA7D-4962-9EC7-5FE6374254C2}" uniqueName="1" name="Peak" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{72AAA502-5133-4DC1-8977-1027DF38D99C}" uniqueName="2" name="Model" queryTableFieldId="2" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{72AAA502-5133-4DC1-8977-1027DF38D99C}" uniqueName="2" name="Model" queryTableFieldId="2" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{0301A6CC-548A-4BB7-9227-3320C06C43F6}" uniqueName="3" name="Center (cm⁻¹)" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{1EB7F6A7-BEE3-4A1E-B044-333891E684A0}" uniqueName="4" name="FWHM (cm⁻¹)" queryTableFieldId="4"/>
     <tableColumn id="5" xr3:uid="{F694254C-9188-4A9A-876A-7FD9EB8C9A0B}" uniqueName="5" name="Area" queryTableFieldId="5"/>
@@ -715,7 +715,7 @@
   <autoFilter ref="B15:G30" xr:uid="{4D14A341-1A1B-417F-A825-A605E9D24775}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{847CD2E0-5A1B-414D-8715-196468A1EE01}" uniqueName="1" name="Peak" queryTableFieldId="1"/>
-    <tableColumn id="2" xr3:uid="{C58BA7AD-B6D5-4264-B175-EA5FA5BC70EB}" uniqueName="2" name="Model" queryTableFieldId="2" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{C58BA7AD-B6D5-4264-B175-EA5FA5BC70EB}" uniqueName="2" name="Model" queryTableFieldId="2" dataDxfId="0"/>
     <tableColumn id="3" xr3:uid="{CF0D7D04-07EB-4125-A990-9932F942A500}" uniqueName="3" name="Center (cm⁻¹)" queryTableFieldId="3"/>
     <tableColumn id="4" xr3:uid="{C450238A-19F9-4921-9FF3-D7B6178D7AB6}" uniqueName="4" name="FWHM (cm⁻¹)" queryTableFieldId="4"/>
     <tableColumn id="5" xr3:uid="{33431B1B-A92E-4213-A6B8-707DB2154302}" uniqueName="5" name="Area" queryTableFieldId="5"/>
@@ -1065,14 +1065,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
       <c r="I2" s="11" t="s">
         <v>24</v>
       </c>
@@ -1095,14 +1095,14 @@
       <c r="Q2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="U2" s="15" t="s">
+      <c r="U2" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="V2" s="16"/>
-      <c r="W2" s="16"/>
-      <c r="X2" s="16"/>
-      <c r="Y2" s="16"/>
-      <c r="Z2" s="17"/>
+      <c r="V2" s="21"/>
+      <c r="W2" s="21"/>
+      <c r="X2" s="21"/>
+      <c r="Y2" s="21"/>
+      <c r="Z2" s="22"/>
     </row>
     <row r="3" spans="2:26" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
@@ -1428,6 +1428,10 @@
     </row>
     <row r="13" spans="2:26" x14ac:dyDescent="0.3">
       <c r="I13" s="12"/>
+      <c r="J13" s="2">
+        <f>(G7-G22)/G7</f>
+        <v>0.2294804678912914</v>
+      </c>
       <c r="L13" s="5"/>
       <c r="M13" s="6"/>
       <c r="N13"/>
@@ -1435,14 +1439,14 @@
       <c r="Q13" s="6"/>
     </row>
     <row r="14" spans="2:26" x14ac:dyDescent="0.3">
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23"/>
       <c r="I14" s="12"/>
       <c r="L14" s="5"/>
       <c r="M14" s="6"/>
@@ -1631,7 +1635,7 @@
       <c r="N21"/>
       <c r="O21" s="5"/>
       <c r="Q21" s="6"/>
-      <c r="T21" s="23" t="s">
+      <c r="T21" s="19" t="s">
         <v>4</v>
       </c>
       <c r="U21" s="2" t="s">
@@ -1665,11 +1669,11 @@
         <f>I22/I7</f>
         <v>1.10255188067483</v>
       </c>
-      <c r="L22" s="19">
+      <c r="L22" s="15">
         <f>SUM(_0_Ne_300_2_5_peak_parameters__420[[#This Row],[Area]])</f>
         <v>9561910018593520</v>
       </c>
-      <c r="M22" s="20">
+      <c r="M22" s="16">
         <f>L22/L7</f>
         <v>0.22220972056817564</v>
       </c>
@@ -1736,11 +1740,11 @@
       <c r="K24" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="L24" s="21">
+      <c r="L24" s="17">
         <f>SUM(F22:F26)</f>
         <v>5.574597375362216E+16</v>
       </c>
-      <c r="M24" s="22">
+      <c r="M24" s="18">
         <f>L24/SUM(Unirradiated_peak_parameters[Area])</f>
         <v>0.31172629711901667</v>
       </c>
@@ -1782,8 +1786,8 @@
       </c>
       <c r="I25" s="12"/>
       <c r="K25" s="1"/>
-      <c r="L25" s="21"/>
-      <c r="M25" s="22">
+      <c r="L25" s="17"/>
+      <c r="M25" s="18">
         <f>L24/I22</f>
         <v>0.28273163610969571</v>
       </c>
@@ -1952,14 +1956,14 @@
       </c>
     </row>
     <row r="33" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B33" s="18" t="s">
+      <c r="B33" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="C33" s="18"/>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
-      <c r="F33" s="18"/>
-      <c r="G33" s="18"/>
+      <c r="C33" s="23"/>
+      <c r="D33" s="23"/>
+      <c r="E33" s="23"/>
+      <c r="F33" s="23"/>
+      <c r="G33" s="23"/>
       <c r="I33" s="12"/>
       <c r="L33" s="5"/>
       <c r="M33" s="6"/>
@@ -2315,14 +2319,14 @@
       <c r="Q47" s="6"/>
     </row>
     <row r="48" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B48" s="18" t="s">
+      <c r="B48" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="C48" s="18"/>
-      <c r="D48" s="18"/>
-      <c r="E48" s="18"/>
-      <c r="F48" s="18"/>
-      <c r="G48" s="18"/>
+      <c r="C48" s="23"/>
+      <c r="D48" s="23"/>
+      <c r="E48" s="23"/>
+      <c r="F48" s="23"/>
+      <c r="G48" s="23"/>
       <c r="I48" s="12"/>
       <c r="L48" s="5"/>
       <c r="M48" s="6"/>
@@ -2846,14 +2850,14 @@
       <c r="Q69" s="14"/>
     </row>
     <row r="70" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B70" s="18" t="s">
+      <c r="B70" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="C70" s="18"/>
-      <c r="D70" s="18"/>
-      <c r="E70" s="18"/>
-      <c r="F70" s="18"/>
-      <c r="G70" s="18"/>
+      <c r="C70" s="23"/>
+      <c r="D70" s="23"/>
+      <c r="E70" s="23"/>
+      <c r="F70" s="23"/>
+      <c r="G70" s="23"/>
       <c r="I70" s="12"/>
       <c r="L70" s="5"/>
       <c r="M70" s="6"/>
@@ -3423,14 +3427,14 @@
       <c r="Q92" s="6"/>
     </row>
     <row r="93" spans="2:17" x14ac:dyDescent="0.3">
-      <c r="B93" s="15" t="s">
+      <c r="B93" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="C93" s="16"/>
-      <c r="D93" s="16"/>
-      <c r="E93" s="16"/>
-      <c r="F93" s="16"/>
-      <c r="G93" s="17"/>
+      <c r="C93" s="21"/>
+      <c r="D93" s="21"/>
+      <c r="E93" s="21"/>
+      <c r="F93" s="21"/>
+      <c r="G93" s="22"/>
       <c r="I93" s="12"/>
       <c r="L93" s="5"/>
       <c r="M93" s="6"/>

</xml_diff>